<commit_message>
feat(divergent-universe): g22-p6-b5 author explicit boss fragment rewards
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions/data/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions/data/DivergentUniverseDecisions.xlsx
@@ -56,7 +56,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'EvolutionOptions'!$A$3:$P$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'CurioVictoryBlessings'!$A$3:$P$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'DomainChoices'!$A$3:$J$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'BattleFragments'!$A$3:$J$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'BattleFragments'!$A$3:$J$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'CurioDomainExpiries'!$A$3:$M$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'CurioBattleStats'!$A$3:$P$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'CurioBattleReactions'!$A$3:$O$8</definedName>
@@ -11151,7 +11151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -11491,7 +11491,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>VersionedProjectPolicy: after each verified won battle, credit the authored fixed base amount for the authenticated domain before separate Curio victory grants and Blessing generation. Combat and Aberration proxies grant 40; Elite proxies grant 100. These amounts are engineering choices, not observed game values: they provide a nonzero repeatable combat income with an explicit higher Elite reward while original drop distributions remain unavailable. Apply the existing global fragment-gain pipeline to this credit independently of each Curio credit. Loss/fault grants nothing, Blessing suppression does not suppress fragments, and no reward RNG is drawn. Result verification, carry, all reward stages and automatic advance roll back together. Do not infer domain from source elite flags, enemy count or account reward displays. No boss policy is declared until that route exists.</t>
+          <t>VersionedProjectPolicy: after each verified won battle, credit the authored fixed base amount for the authenticated domain before separate Curio victory grants and Blessing generation. Combat and Aberration proxies grant 40; Elite proxies grant 100. These amounts are engineering choices, not observed game values: they provide a nonzero repeatable combat income with an explicit higher Elite reward while original drop distributions remain unavailable. Apply the existing global fragment-gain pipeline to this credit independently of each Curio credit. Loss/fault grants nothing, Blessing suppression does not suppress fragments, and no reward RNG is drawn. Result verification, carry, all reward stages and automatic advance roll back together. Do not infer domain from source elite flags, enemy count or account reward displays. Boss uses a separate explicit-policy row without enlarging the legacy three-label domain-choice route.</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
@@ -11531,7 +11531,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>VersionedProjectPolicy: after each verified won battle, credit the authored fixed base amount for the authenticated domain before separate Curio victory grants and Blessing generation. Combat and Aberration proxies grant 40; Elite proxies grant 100. These amounts are engineering choices, not observed game values: they provide a nonzero repeatable combat income with an explicit higher Elite reward while original drop distributions remain unavailable. Apply the existing global fragment-gain pipeline to this credit independently of each Curio credit. Loss/fault grants nothing, Blessing suppression does not suppress fragments, and no reward RNG is drawn. Result verification, carry, all reward stages and automatic advance roll back together. Do not infer domain from source elite flags, enemy count or account reward displays. No boss policy is declared until that route exists.</t>
+          <t>VersionedProjectPolicy: after each verified won battle, credit the authored fixed base amount for the authenticated domain before separate Curio victory grants and Blessing generation. Combat and Aberration proxies grant 40; Elite proxies grant 100. These amounts are engineering choices, not observed game values: they provide a nonzero repeatable combat income with an explicit higher Elite reward while original drop distributions remain unavailable. Apply the existing global fragment-gain pipeline to this credit independently of each Curio credit. Loss/fault grants nothing, Blessing suppression does not suppress fragments, and no reward RNG is drawn. Result verification, carry, all reward stages and automatic advance roll back together. Do not infer domain from source elite flags, enemy count or account reward displays. Boss uses a separate explicit-policy row without enlarging the legacy three-label domain-choice route.</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
@@ -11571,7 +11571,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>VersionedProjectPolicy: after each verified won battle, credit the authored fixed base amount for the authenticated domain before separate Curio victory grants and Blessing generation. Combat and Aberration proxies grant 40; Elite proxies grant 100. These amounts are engineering choices, not observed game values: they provide a nonzero repeatable combat income with an explicit higher Elite reward while original drop distributions remain unavailable. Apply the existing global fragment-gain pipeline to this credit independently of each Curio credit. Loss/fault grants nothing, Blessing suppression does not suppress fragments, and no reward RNG is drawn. Result verification, carry, all reward stages and automatic advance roll back together. Do not infer domain from source elite flags, enemy count or account reward displays. No boss policy is declared until that route exists.</t>
+          <t>VersionedProjectPolicy: after each verified won battle, credit the authored fixed base amount for the authenticated domain before separate Curio victory grants and Blessing generation. Combat and Aberration proxies grant 40; Elite proxies grant 100. These amounts are engineering choices, not observed game values: they provide a nonzero repeatable combat income with an explicit higher Elite reward while original drop distributions remain unavailable. Apply the existing global fragment-gain pipeline to this credit independently of each Curio credit. Loss/fault grants nothing, Blessing suppression does not suppress fragments, and no reward RNG is drawn. Result verification, carry, all reward stages and automatic advance roll back together. Do not infer domain from source elite flags, enemy count or account reward displays. Boss uses a separate explicit-policy row without enlarging the legacy three-label domain-choice route.</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
@@ -11586,8 +11586,48 @@
       </c>
       <c r="J10" s="9" t="n"/>
     </row>
+    <row r="11">
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>du.battle-fragments.boss</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>FixedVerifiedDomainCredit</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>VersionedProjectPolicy: credit 100 base fragments after a verified win in an explicitly bound Boss reward domain, before separate Curio victory grants, battle lifetimes and the existing provisional Blessing offer. This is an engineering choice, not an observed game amount or a claim of original Boss eligibility, AI, phases or drops. Use the same nonzero base as the existing Elite proxy to extend the bounded reward pipeline without inventing a higher Boss multiplier; the domains remain independently replaceable. Select the domain only from the immutable room binding, never from preset level, stage elite flags or an adapter label. Apply current global fragment-gain modifiers to this credit separately from each Curio credit. Loss/fault grants nothing; Blessing suppression does not suppress fragments; the fixed base draws no RNG. Verified result, carry, all grants and next-node initialization commit or roll back together. The three-label legacy domain-choice route remains unchanged.</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Replace Boss amount, fixed versus random distribution, per-battle versus per-enemy timing, difficulty scaling, base Blessing pool and reward ordering independently when released current-profile drop programs or reproducible observations establish them. Alternatives are a zero Boss base, a larger Boss-specific constant or integer range sampling; none is proven by the inspected constants, source labels or public domain overview. This explicit 100-fragment policy has low parity confidence, preserves independent Boss-domain authentication, and must not terminalize original Boss programs or source obligations.</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>14|24|41|66</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:J10"/>
+  <autoFilter ref="A3:J11"/>
   <dataValidations count="4">
     <dataValidation sqref="B8:B1007" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." type="whole">
       <formula1>1</formula1>

</xml_diff>

<commit_message>
feat(divergent-universe): g22-p5-b2 execute sapient pen effects
Bind policy-reviewed Basic/Skill Punchline gains and timed Elation bonuses through shared Rule IR. Exclude linked entities independently of presence, preserve recipient-scoped effects, and share checked keyed-resource event arithmetic.

Include production workbook/Sora output, native regressions, current RNG vectors, generated inventory and state documentation. Verified affected package tests, workspace tests, Clippy, formatting, source checks and workbook drift/visual QA. Full-run and remaining Elation lifecycle coverage remain pending.
</commit_message>
<xml_diff>
--- a/config/divergent-universe-decisions/data/DivergentUniverseDecisions.xlsx
+++ b/config/divergent-universe-decisions/data/DivergentUniverseDecisions.xlsx
@@ -35753,8 +35753,8 @@
     <col width="28" customWidth="1" style="5" min="13" max="13"/>
     <col width="28" customWidth="1" style="5" min="14" max="14"/>
     <col width="28" customWidth="1" style="5" min="15" max="15"/>
-    <col width="28" customWidth="1" style="5" min="16" max="16"/>
-    <col width="28" customWidth="1" style="5" min="17" max="17"/>
+    <col width="90" customWidth="1" style="5" min="16" max="16"/>
+    <col width="90" customWidth="1" style="5" min="17" max="17"/>
     <col width="28" customWidth="1" style="5" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -36298,7 +36298,7 @@
       <c r="Q7" s="6" t="n"/>
       <c r="R7" s="6" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="260" customHeight="1">
       <c r="A8" s="9" t="n"/>
       <c r="B8" s="9" t="n">
         <v>1</v>
@@ -36360,12 +36360,12 @@
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>VersionedProjectPolicy, authored but not yet executed: original party combat forms determine Path membership; any original Elation party form satisfies presence, including a defeated member. Eligible original non-Elation owners trigger at ActionResolved AfterAction, priority zero, once per action for Basic or Skill regardless of Attack tag or hit count. Grant two to the side's single shared.punchline binding, then apply one dispellable additive StatKind::Elation bonus of 0.5 to each living/present original Elation recipient in formation order. TargetTurnEnd duration two, replace and refresh across casters rather than stack; no Ultimate, follow-up, summon, memosprite or shared-actor trigger. No RNG or Activity mutation. Shared-meter initial value, maximum, overflow and wave/battle carry belong to the separate BattleTeamResources assembly policy, not Curio operands or defaults; implementing the meter does not implement this Curio.</t>
+          <t>VersionedProjectPolicy: original party combat forms determine Path membership; any original Elation party form satisfies presence, including a defeated member. Eligible original non-Elation owners trigger at ActionResolved AfterAction, priority zero, once per action for Basic or Skill regardless of Attack tag or hit count. Grant two to the side's single shared.punchline binding, then apply one dispellable additive StatKind::Elation bonus of 0.5 to each living/present original Elation recipient in formation order. TargetTurnEnd duration two, replace and refresh across casters rather than stack. Recipient-scoped persistence survives provider defeat and waves until expiry or dispel. No Ultimate, follow-up, summon, memosprite or shared-actor trigger. No RNG or Activity mutation. Shared-meter initial value, maximum, overflow and wave/battle carry belong to the separate BattleTeamResources assembly policy, not Curio operands or defaults. Character Skill resource deltas and Aha/Certified Banger lifecycle are separate unimplemented boundaries.</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Low confidence for party presence while defeated, original-form membership, action observation point, cause ownership, ordering, dispel and cross-caster refresh. Bounded 2026-10-02 public cross-check: https://honkai-star-rail.fandom.com/wiki/Sapient_Pen confirms only the current Arcadian Chronicles player-facing clauses, not hidden scheduling; its older Quantum/Wind variant is excluded. Alternatives: active-only presence, per-hit triggers, caster-specific stacking, nondispellable bonus and source-turn duration. Data tests weighted_curio_elation validate exact operands, joins, policy labels and all four sources; they do not prove battle execution. Replace fields independently when released StageAbility_633415 or reproducible current observations establish trigger/recipient/refresh semantics. Runtime admission still requires real-command fixtures for both run families and explicit shared-meter assembly, overflow, lifecycle and reconstruction tests.</t>
+          <t>Low confidence for party presence while defeated, original-form membership, action observation point, cause ownership, ordering, dispel and cross-caster refresh. Bounded 2026-10-02 public cross-check: https://honkai-star-rail.fandom.com/wiki/Sapient_Pen confirms only the current Arcadian Chronicles player-facing clauses, not hidden scheduling; its older Quantum/Wind variant is excluded. Alternatives: active-only presence, per-hit triggers, caster-specific stacking, nondispellable bonus and source-turn duration. Data tests weighted_curio_elation validate exact operands, joins, policy labels and all four sources; they do not prove battle execution. Mode fixtures weighted_curio_elation separately execute real commands in both run families and controlled resource/stat/lifecycle/reconstruction boundaries. Replace fields independently when released StageAbility_633415 or reproducible current observations establish trigger/recipient/refresh semantics. Forge offer/slot admission and full-run release coverage remain pending.</t>
         </is>
       </c>
       <c r="R8" s="9" t="inlineStr">

</xml_diff>